<commit_message>
Cap nhat du lieu - 08/05/2026  8:49
</commit_message>
<xml_diff>
--- a/database_cong_trinh.xlsx
+++ b/database_cong_trinh.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sửa chữa lớn TSCĐ thay thế LBFCO,FCO,LA ngăn ngừa sự cố 2026</t>
+          <t>Sửa chữa lớn TSCĐ thay thế LBFCO, FCO, LA... ngăn ngừa sự cố năm 2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Sửa chữa nhà đặt MPĐ, nhà máy An Hội, Đặc khu công đảo</t>
+          <t>Sửa chữa nhà đặt máy phát điện, nhà máy An Hội, Đặc khu Côn Đảo</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4250,7 +4250,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SCL Hệ thống điện bằng biện pháp Live-Line 2026</t>
+          <t>Sửa chữa lớn hệ thống điện bằng biện pháp Live-Line năm 2026</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>SCL Công Xa Công ty Điện lực Vũng Tàu 2026</t>
+          <t>Sửa chữa lớn công xa Công ty Điện lực Vũng Tàu năm 2026</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Sửa chữa lớn Công xa 2026</t>
+          <t>Sửa chữa lớn công xa Công ty Điện lực Vũng Tàu năm 2026</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -12022,7 +12022,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>SCL MPĐ Cummins G1,G2 NMĐ An Hội 2026</t>
+          <t>Sửa chữa lớn máy phát điện Cummins G1, G2 nhà máy điện An hội năm 2026</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -14000,7 +14000,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Sửa chữa lớn Công xa 2026</t>
+          <t>Sửa chữa lớn công xa Công ty Điện lực Vũng Tàu năm 2026</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -15978,7 +15978,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Sửa chữa lớn TSCĐ thay thế LBFCO,FCO,LA ngăn ngừa sự cố 2026</t>
+          <t>Sửa chữa lớn TSCĐ thay thế LBFCO, FCO, LA... ngăn ngừa sự cố năm 2026</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -20086,7 +20086,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>SCL Hệ thống điện bằng biện pháp Live-Line 2026</t>
+          <t>Sửa chữa lớn hệ thống điện bằng biện pháp Live-Line năm 2026</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
@@ -22216,7 +22216,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>SCL Đường dây và trạm biến áp năm 2026</t>
+          <t>Sửa chữa lớn đường dây trung, hạ thế và trạm biến áp năm 2026</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">

</xml_diff>